<commit_message>
IPC applicable on reports
</commit_message>
<xml_diff>
--- a/app/templates/report/reservaslau.xlsx
+++ b/app/templates/report/reservaslau.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1E9870F-C69B-471E-9E5A-DE9B642DAF88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65214E50-C4AB-4528-AF1A-0D5ADC81F9D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Reservas" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Reservas!$A$3:$AK$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Reservas!$A$3:$AL$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="48">
   <si>
     <t>Reservas LAU y otras</t>
   </si>
@@ -179,6 +179,9 @@
   </si>
   <si>
     <t>Código SAP</t>
+  </si>
+  <si>
+    <t>Aplica IPC?</t>
   </si>
 </sst>
 </file>
@@ -299,7 +302,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -333,6 +336,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -717,7 +721,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AK4"/>
+  <dimension ref="A1:AL4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="1" bestFit="1" customWidth="1"/>
@@ -731,18 +735,18 @@
     <col min="9" max="11" width="12" style="1" customWidth="1"/>
     <col min="12" max="12" width="25" style="1" customWidth="1"/>
     <col min="13" max="14" width="17.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="23" width="12.5546875" style="1" customWidth="1"/>
-    <col min="24" max="24" width="12" style="1" customWidth="1"/>
-    <col min="25" max="25" width="23.44140625" style="1" customWidth="1"/>
-    <col min="26" max="30" width="12" style="1" customWidth="1"/>
-    <col min="31" max="34" width="14.33203125" style="1" customWidth="1"/>
-    <col min="35" max="35" width="12.5546875" style="1" customWidth="1"/>
-    <col min="36" max="36" width="32.33203125" style="1" customWidth="1"/>
-    <col min="37" max="37" width="59.6640625" style="1" customWidth="1"/>
-    <col min="38" max="16384" width="14.44140625" style="1"/>
+    <col min="15" max="24" width="12.5546875" style="1" customWidth="1"/>
+    <col min="25" max="25" width="12" style="1" customWidth="1"/>
+    <col min="26" max="26" width="23.44140625" style="1" customWidth="1"/>
+    <col min="27" max="31" width="12" style="1" customWidth="1"/>
+    <col min="32" max="35" width="14.33203125" style="1" customWidth="1"/>
+    <col min="36" max="36" width="12.5546875" style="1" customWidth="1"/>
+    <col min="37" max="37" width="32.33203125" style="1" customWidth="1"/>
+    <col min="38" max="38" width="59.6640625" style="1" customWidth="1"/>
+    <col min="39" max="16384" width="14.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -757,10 +761,7 @@
         <f>SUBTOTAL(9,O4:O99999)</f>
         <v>0</v>
       </c>
-      <c r="R1" s="16">
-        <f>SUBTOTAL(9,R4:R99999)</f>
-        <v>0</v>
-      </c>
+      <c r="P1" s="17"/>
       <c r="S1" s="16">
         <f>SUBTOTAL(9,S4:S99999)</f>
         <v>0</v>
@@ -769,24 +770,24 @@
         <f>SUBTOTAL(9,T4:T99999)</f>
         <v>0</v>
       </c>
-      <c r="V1" s="16">
-        <f>SUBTOTAL(9,V4:V99999)</f>
-        <v>0</v>
-      </c>
-      <c r="X1" s="16">
-        <f>SUBTOTAL(9,X4:X99999)</f>
-        <v>0</v>
-      </c>
-      <c r="Z1" s="16">
-        <f>SUBTOTAL(9,Z4:Z99999)</f>
+      <c r="U1" s="16">
+        <f>SUBTOTAL(9,U4:U99999)</f>
+        <v>0</v>
+      </c>
+      <c r="W1" s="16">
+        <f>SUBTOTAL(9,W4:W99999)</f>
+        <v>0</v>
+      </c>
+      <c r="Y1" s="16">
+        <f>SUBTOTAL(9,Y4:Y99999)</f>
         <v>0</v>
       </c>
       <c r="AA1" s="16">
         <f>SUBTOTAL(9,AA4:AA99999)</f>
         <v>0</v>
       </c>
-      <c r="AF1" s="16">
-        <f>SUBTOTAL(9,AF4:AF99999)</f>
+      <c r="AB1" s="16">
+        <f>SUBTOTAL(9,AB4:AB99999)</f>
         <v>0</v>
       </c>
       <c r="AG1" s="16">
@@ -797,8 +798,12 @@
         <f>SUBTOTAL(9,AH4:AH99999)</f>
         <v>0</v>
       </c>
+      <c r="AI1" s="16">
+        <f>SUBTOTAL(9,AI4:AI99999)</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -824,40 +829,41 @@
       </c>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
-      <c r="R2" s="3" t="s">
+      <c r="R2" s="4"/>
+      <c r="S2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
-      <c r="V2" s="4" t="s">
+      <c r="V2" s="3"/>
+      <c r="W2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="W2" s="4"/>
-      <c r="X2" s="3" t="s">
+      <c r="X2" s="4"/>
+      <c r="Y2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Y2" s="3"/>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
-      <c r="AB2" s="4" t="s">
+      <c r="AB2" s="3"/>
+      <c r="AC2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="AC2" s="4"/>
       <c r="AD2" s="4"/>
-      <c r="AE2" s="3" t="s">
+      <c r="AE2" s="4"/>
+      <c r="AF2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3"/>
       <c r="AI2" s="3"/>
       <c r="AJ2" s="3"/>
-      <c r="AK2" s="4" t="s">
+      <c r="AK2" s="3"/>
+      <c r="AL2" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:37" s="11" customFormat="1" ht="25.2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:38" s="11" customFormat="1" ht="25.2" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>8</v>
       </c>
@@ -904,73 +910,76 @@
         <v>3</v>
       </c>
       <c r="P3" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q3" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="Q3" s="10" t="s">
+      <c r="R3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="R3" s="9" t="s">
+      <c r="S3" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="S3" s="9" t="s">
+      <c r="T3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="T3" s="9" t="s">
+      <c r="U3" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="U3" s="9" t="s">
+      <c r="V3" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="V3" s="10" t="s">
+      <c r="W3" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="W3" s="10" t="s">
+      <c r="X3" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="X3" s="9" t="s">
+      <c r="Y3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="Y3" s="9" t="s">
+      <c r="Z3" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="Z3" s="9" t="s">
+      <c r="AA3" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="AA3" s="9" t="s">
+      <c r="AB3" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="AB3" s="10" t="s">
+      <c r="AC3" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="AC3" s="10" t="s">
+      <c r="AD3" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="AD3" s="10" t="s">
+      <c r="AE3" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="AE3" s="9" t="s">
+      <c r="AF3" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="AF3" s="9" t="s">
+      <c r="AG3" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="AG3" s="9" t="s">
+      <c r="AH3" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="AH3" s="9" t="s">
+      <c r="AI3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="AI3" s="9" t="s">
+      <c r="AJ3" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="AJ3" s="9" t="s">
+      <c r="AK3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="AK3" s="10" t="s">
+      <c r="AL3" s="10" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -992,21 +1001,21 @@
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
       <c r="O4" s="7"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="13" t="s">
+      <c r="P4" s="7"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="R4" s="7"/>
       <c r="S4" s="7"/>
-      <c r="T4" s="12"/>
-      <c r="U4" s="13" t="s">
+      <c r="T4" s="7"/>
+      <c r="U4" s="12"/>
+      <c r="V4" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="V4" s="7"/>
-      <c r="W4" s="13" t="s">
+      <c r="W4" s="7"/>
+      <c r="X4" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="X4" s="7"/>
       <c r="Y4" s="7"/>
       <c r="Z4" s="7"/>
       <c r="AA4" s="7"/>
@@ -1017,14 +1026,15 @@
       <c r="AF4" s="7"/>
       <c r="AG4" s="7"/>
       <c r="AH4" s="7"/>
-      <c r="AI4" s="13" t="s">
+      <c r="AI4" s="7"/>
+      <c r="AJ4" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="AJ4" s="5"/>
-      <c r="AK4" s="7"/>
+      <c r="AK4" s="5"/>
+      <c r="AL4" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:AK3" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A3:AL3" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>

</xml_diff>